<commit_message>
Simplify monthly equipment report
</commit_message>
<xml_diff>
--- a/outputs/modele_base_heures_engins.xlsx
+++ b/outputs/modele_base_heures_engins.xlsx
@@ -2,10 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UTILISATEURS" sheetId="1" r:id="R8a98ef6cc6e241df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ENGINS" sheetId="2" r:id="R7e6ac65109e64964"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RELEVES" sheetId="3" r:id="R1068924f8df84f34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VALIDATIONS" sheetId="4" r:id="R2f8eec144e014082"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONDUCTEURS" sheetId="1" r:id="R7a06c2c5413a465c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RELEVES_MENSUELS" sheetId="2" r:id="R768d8df1903a42b2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -212,139 +210,19 @@
         <x:v>ID</x:v>
       </x:c>
       <x:c r="B1" s="2" t="str">
+        <x:v>NOM</x:v>
+      </x:c>
+      <x:c r="C1" s="2" t="str">
+        <x:v>PRENOM</x:v>
+      </x:c>
+      <x:c r="D1" s="2" t="str">
         <x:v>PIN</x:v>
-      </x:c>
-      <x:c r="C1" s="2" t="str">
-        <x:v>NOM</x:v>
-      </x:c>
-      <x:c r="D1" s="2" t="str">
-        <x:v>PRENOM</x:v>
       </x:c>
       <x:c r="E1" s="2" t="str">
         <x:v>ROLE</x:v>
       </x:c>
       <x:c r="F1" s="2" t="str">
         <x:v>ACTIF</x:v>
-      </x:c>
-      <x:c r="G1" s="2" t="str">
-        <x:v>COMMENTAIRE</x:v>
-      </x:c>
-      <x:c r="H1" s="2"/>
-      <x:c r="I1" s="2"/>
-      <x:c r="J1" s="2"/>
-      <x:c r="K1" s="2"/>
-      <x:c r="L1" s="2"/>
-      <x:c r="M1" s="2"/>
-      <x:c r="N1" s="2"/>
-      <x:c r="O1" s="2"/>
-      <x:c r="P1" s="2"/>
-      <x:c r="Q1" s="2"/>
-      <x:c r="R1" s="2"/>
-      <x:c r="S1" s="2"/>
-      <x:c r="T1" s="2"/>
-      <x:c r="U1" s="2"/>
-      <x:c r="V1" s="2"/>
-      <x:c r="W1" s="2"/>
-      <x:c r="X1" s="2"/>
-      <x:c r="Y1" s="2"/>
-      <x:c r="Z1" s="2"/>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" t="str">
-        <x:v>COND001</x:v>
-      </x:c>
-      <x:c r="B2" t="str">
-        <x:v>1234</x:v>
-      </x:c>
-      <x:c r="C2" t="str">
-        <x:v>Dupont</x:v>
-      </x:c>
-      <x:c r="D2" t="str">
-        <x:v>Jean</x:v>
-      </x:c>
-      <x:c r="E2" t="str">
-        <x:v>conducteur</x:v>
-      </x:c>
-      <x:c r="F2" t="str">
-        <x:v>OUI</x:v>
-      </x:c>
-      <x:c r="G2" t="str">
-        <x:v>Exemple conducteur</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" t="str">
-        <x:v>COND002</x:v>
-      </x:c>
-      <x:c r="B3" t="str">
-        <x:v>2345</x:v>
-      </x:c>
-      <x:c r="C3" t="str">
-        <x:v>Martin</x:v>
-      </x:c>
-      <x:c r="D3" t="str">
-        <x:v>Sophie</x:v>
-      </x:c>
-      <x:c r="E3" t="str">
-        <x:v>conducteur</x:v>
-      </x:c>
-      <x:c r="F3" t="str">
-        <x:v>OUI</x:v>
-      </x:c>
-      <x:c r="G3" t="str">
-        <x:v>Exemple conducteur</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" t="str">
-        <x:v>RESP001</x:v>
-      </x:c>
-      <x:c r="B4" t="str">
-        <x:v>9999</x:v>
-      </x:c>
-      <x:c r="C4" t="str">
-        <x:v>Responsable</x:v>
-      </x:c>
-      <x:c r="D4" t="str">
-        <x:v>Travaux</x:v>
-      </x:c>
-      <x:c r="E4" t="str">
-        <x:v>responsable</x:v>
-      </x:c>
-      <x:c r="F4" t="str">
-        <x:v>OUI</x:v>
-      </x:c>
-      <x:c r="G4" t="str">
-        <x:v>Compte responsable</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="2" t="str">
-        <x:v>ID_ENGIN</x:v>
-      </x:c>
-      <x:c r="B1" s="2" t="str">
-        <x:v>DESIGNATION</x:v>
-      </x:c>
-      <x:c r="C1" s="2" t="str">
-        <x:v>IMMATRICULATION</x:v>
-      </x:c>
-      <x:c r="D1" s="2" t="str">
-        <x:v>TYPE</x:v>
-      </x:c>
-      <x:c r="E1" s="2" t="str">
-        <x:v>ACTIF</x:v>
-      </x:c>
-      <x:c r="F1" s="2" t="str">
-        <x:v>COMMENTAIRE</x:v>
       </x:c>
       <x:c r="G1" s="2"/>
       <x:c r="H1" s="2"/>
@@ -368,93 +246,123 @@
       <x:c r="Z1" s="2"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" t="str">
-        <x:v>PELLE001</x:v>
+      <x:c r="A2" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>Pelle 8T</x:v>
-      </x:c>
-      <x:c r="C2" t="str"/>
-      <x:c r="D2" t="str">
-        <x:v>Pelle</x:v>
+        <x:v>BAOUZ</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>JULIEN</x:v>
+      </x:c>
+      <x:c r="D2" t="n">
+        <x:v>3960</x:v>
       </x:c>
       <x:c r="E2" t="str">
-        <x:v>OUI</x:v>
+        <x:v>employe</x:v>
       </x:c>
       <x:c r="F2" t="str">
-        <x:v>Exemple</x:v>
+        <x:v>OUI</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" t="str">
-        <x:v>CHARGEUR001</x:v>
+      <x:c r="A3" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Chargeur</x:v>
-      </x:c>
-      <x:c r="C3" t="str"/>
-      <x:c r="D3" t="str">
-        <x:v>Chargeur</x:v>
+        <x:v>LANGE</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>DAVID</x:v>
+      </x:c>
+      <x:c r="D3" t="n">
+        <x:v>5678</x:v>
       </x:c>
       <x:c r="E3" t="str">
-        <x:v>OUI</x:v>
+        <x:v>responsable</x:v>
       </x:c>
       <x:c r="F3" t="str">
-        <x:v>Exemple</x:v>
+        <x:v>OUI</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" t="str">
-        <x:v>MINI001</x:v>
+      <x:c r="A4" t="n">
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>Mini-pelle</x:v>
-      </x:c>
-      <x:c r="C4" t="str"/>
-      <x:c r="D4" t="str">
-        <x:v>Mini-pelle</x:v>
+        <x:v>BOUCHEROT</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>REMY</x:v>
+      </x:c>
+      <x:c r="D4" t="n">
+        <x:v>5412</x:v>
       </x:c>
       <x:c r="E4" t="str">
-        <x:v>OUI</x:v>
+        <x:v>employe</x:v>
       </x:c>
       <x:c r="F4" t="str">
-        <x:v>Exemple</x:v>
+        <x:v>OUI</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" t="str">
-        <x:v>CAMION001</x:v>
+      <x:c r="A5" t="n">
+        <x:v>4</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Camion benne</x:v>
-      </x:c>
-      <x:c r="C5" t="str"/>
-      <x:c r="D5" t="str">
-        <x:v>Camion</x:v>
+        <x:v>NOM EMPLOYE 3</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>YVAN</x:v>
+      </x:c>
+      <x:c r="D5" t="n">
+        <x:v>6875</x:v>
       </x:c>
       <x:c r="E5" t="str">
-        <x:v>OUI</x:v>
+        <x:v>employe</x:v>
       </x:c>
       <x:c r="F5" t="str">
-        <x:v>Exemple</x:v>
+        <x:v>OUI</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" t="str">
-        <x:v>COMPACT001</x:v>
+      <x:c r="A6" t="n">
+        <x:v>5</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Compacteur</x:v>
-      </x:c>
-      <x:c r="C6" t="str"/>
-      <x:c r="D6" t="str">
-        <x:v>Compacteur</x:v>
+        <x:v>NOM EMPLOYE 4</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>YACIN</x:v>
+      </x:c>
+      <x:c r="D6" t="n">
+        <x:v>5143</x:v>
       </x:c>
       <x:c r="E6" t="str">
-        <x:v>OUI</x:v>
+        <x:v>employe</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>Exemple</x:v>
+        <x:v>OUI</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>PHAN</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>HUGO</x:v>
+      </x:c>
+      <x:c r="D7" t="n">
+        <x:v>8732</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>employe</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>OUI</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -462,7 +370,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
@@ -474,98 +382,41 @@
         <x:v>TIMESTAMP</x:v>
       </x:c>
       <x:c r="C1" s="2" t="str">
+        <x:v>MOIS</x:v>
+      </x:c>
+      <x:c r="D1" s="2" t="str">
         <x:v>ID_CONDUCTEUR</x:v>
       </x:c>
-      <x:c r="D1" s="2" t="str">
+      <x:c r="E1" s="2" t="str">
         <x:v>NOM</x:v>
       </x:c>
-      <x:c r="E1" s="2" t="str">
+      <x:c r="F1" s="2" t="str">
         <x:v>PRENOM</x:v>
       </x:c>
-      <x:c r="F1" s="2" t="str">
-        <x:v>SEMAINE_DU</x:v>
-      </x:c>
       <x:c r="G1" s="2" t="str">
-        <x:v>SEMAINE_AU</x:v>
+        <x:v>ROLE</x:v>
       </x:c>
       <x:c r="H1" s="2" t="str">
-        <x:v>ORDRE</x:v>
+        <x:v>SITE</x:v>
       </x:c>
       <x:c r="I1" s="2" t="str">
-        <x:v>JOUR</x:v>
+        <x:v>DATE_RELEVE</x:v>
       </x:c>
       <x:c r="J1" s="2" t="str">
-        <x:v>DATE</x:v>
+        <x:v>IMMATRICULATION</x:v>
       </x:c>
       <x:c r="K1" s="2" t="str">
-        <x:v>ENGIN</x:v>
+        <x:v>HEURE_PORTEUR</x:v>
       </x:c>
       <x:c r="L1" s="2" t="str">
-        <x:v>CHANTIER</x:v>
+        <x:v>HEURE_AUXILIAIRES</x:v>
       </x:c>
       <x:c r="M1" s="2" t="str">
-        <x:v>CONDUCTEUR</x:v>
+        <x:v>KILOMETRAGE</x:v>
       </x:c>
       <x:c r="N1" s="2" t="str">
-        <x:v>COMPTEUR_DEBUT</x:v>
-      </x:c>
-      <x:c r="O1" s="2" t="str">
-        <x:v>COMPTEUR_FIN</x:v>
-      </x:c>
-      <x:c r="P1" s="2" t="str">
-        <x:v>TOTAL_HEURES</x:v>
-      </x:c>
-      <x:c r="Q1" s="2" t="str">
-        <x:v>GAZOLE_L</x:v>
-      </x:c>
-      <x:c r="R1" s="2" t="str">
-        <x:v>OBSERVATIONS</x:v>
-      </x:c>
-      <x:c r="S1" s="2"/>
-      <x:c r="T1" s="2"/>
-      <x:c r="U1" s="2"/>
-      <x:c r="V1" s="2"/>
-      <x:c r="W1" s="2"/>
-      <x:c r="X1" s="2"/>
-      <x:c r="Y1" s="2"/>
-      <x:c r="Z1" s="2"/>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="2" t="str">
-        <x:v>ID_CONDUCTEUR</x:v>
-      </x:c>
-      <x:c r="B1" s="2" t="str">
-        <x:v>SEMAINE_DU</x:v>
-      </x:c>
-      <x:c r="C1" s="2" t="str">
-        <x:v>VISA_CONDUCTEUR</x:v>
-      </x:c>
-      <x:c r="D1" s="2" t="str">
-        <x:v>DATE_VISA_CONDUCTEUR</x:v>
-      </x:c>
-      <x:c r="E1" s="2" t="str">
-        <x:v>VISA_RESPONSABLE</x:v>
-      </x:c>
-      <x:c r="F1" s="2" t="str">
-        <x:v>DATE_VISA_RESPONSABLE</x:v>
-      </x:c>
-      <x:c r="G1" s="2"/>
-      <x:c r="H1" s="2"/>
-      <x:c r="I1" s="2"/>
-      <x:c r="J1" s="2"/>
-      <x:c r="K1" s="2"/>
-      <x:c r="L1" s="2"/>
-      <x:c r="M1" s="2"/>
-      <x:c r="N1" s="2"/>
+        <x:v>COMMENTAIRE</x:v>
+      </x:c>
       <x:c r="O1" s="2"/>
       <x:c r="P1" s="2"/>
       <x:c r="Q1" s="2"/>

</xml_diff>

<commit_message>
Add audit and responsible reporting
</commit_message>
<xml_diff>
--- a/outputs/modele_base_heures_engins.xlsx
+++ b/outputs/modele_base_heures_engins.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONDUCTEURS" sheetId="1" r:id="R7a06c2c5413a465c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RELEVES_MENSUELS" sheetId="2" r:id="R768d8df1903a42b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONDUCTEURS" sheetId="1" r:id="Rfabcd3aebfc54f09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RELEVES_MENSUELS" sheetId="2" r:id="R27805e7f03124b89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AUDIT" sheetId="3" r:id="Re75749e516704d66"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -224,7 +225,9 @@
       <x:c r="F1" s="2" t="str">
         <x:v>ACTIF</x:v>
       </x:c>
-      <x:c r="G1" s="2"/>
+      <x:c r="G1" s="2" t="str">
+        <x:v>EMAIL</x:v>
+      </x:c>
       <x:c r="H1" s="2"/>
       <x:c r="I1" s="2"/>
       <x:c r="J1" s="2"/>
@@ -264,6 +267,7 @@
       <x:c r="F2" t="str">
         <x:v>OUI</x:v>
       </x:c>
+      <x:c r="G2" t="str"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="n">
@@ -284,6 +288,7 @@
       <x:c r="F3" t="str">
         <x:v>OUI</x:v>
       </x:c>
+      <x:c r="G3" t="str"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="n">
@@ -304,6 +309,7 @@
       <x:c r="F4" t="str">
         <x:v>OUI</x:v>
       </x:c>
+      <x:c r="G4" t="str"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="n">
@@ -324,6 +330,7 @@
       <x:c r="F5" t="str">
         <x:v>OUI</x:v>
       </x:c>
+      <x:c r="G5" t="str"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="n">
@@ -344,6 +351,7 @@
       <x:c r="F6" t="str">
         <x:v>OUI</x:v>
       </x:c>
+      <x:c r="G6" t="str"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="n">
@@ -364,6 +372,7 @@
       <x:c r="F7" t="str">
         <x:v>OUI</x:v>
       </x:c>
+      <x:c r="G7" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -433,4 +442,59 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="2" t="str">
+        <x:v>ID_AUDIT</x:v>
+      </x:c>
+      <x:c r="B1" s="2" t="str">
+        <x:v>TIMESTAMP</x:v>
+      </x:c>
+      <x:c r="C1" s="2" t="str">
+        <x:v>ACTION</x:v>
+      </x:c>
+      <x:c r="D1" s="2" t="str">
+        <x:v>ID_UTILISATEUR</x:v>
+      </x:c>
+      <x:c r="E1" s="2" t="str">
+        <x:v>NOM</x:v>
+      </x:c>
+      <x:c r="F1" s="2" t="str">
+        <x:v>PRENOM</x:v>
+      </x:c>
+      <x:c r="G1" s="2" t="str">
+        <x:v>ROLE</x:v>
+      </x:c>
+      <x:c r="H1" s="2" t="str">
+        <x:v>DETAILS</x:v>
+      </x:c>
+      <x:c r="I1" s="2" t="str">
+        <x:v>USER_AGENT</x:v>
+      </x:c>
+      <x:c r="J1" s="2"/>
+      <x:c r="K1" s="2"/>
+      <x:c r="L1" s="2"/>
+      <x:c r="M1" s="2"/>
+      <x:c r="N1" s="2"/>
+      <x:c r="O1" s="2"/>
+      <x:c r="P1" s="2"/>
+      <x:c r="Q1" s="2"/>
+      <x:c r="R1" s="2"/>
+      <x:c r="S1" s="2"/>
+      <x:c r="T1" s="2"/>
+      <x:c r="U1" s="2"/>
+      <x:c r="V1" s="2"/>
+      <x:c r="W1" s="2"/>
+      <x:c r="X1" s="2"/>
+      <x:c r="Y1" s="2"/>
+      <x:c r="Z1" s="2"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Ajoute lien app aux emails responsables
</commit_message>
<xml_diff>
--- a/outputs/modele_base_heures_engins.xlsx
+++ b/outputs/modele_base_heures_engins.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONDUCTEURS" sheetId="1" r:id="Rfabcd3aebfc54f09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RELEVES_MENSUELS" sheetId="2" r:id="R27805e7f03124b89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AUDIT" sheetId="3" r:id="Re75749e516704d66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONDUCTEURS" sheetId="1" r:id="R2beb8f7a4738418a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RELEVES_MENSUELS" sheetId="2" r:id="Rae7dca00587e409f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AUDIT" sheetId="3" r:id="R1b9e2465322e4b6c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -374,6 +374,25 @@
       </x:c>
       <x:c r="G7" t="str"/>
     </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>FOURNIER</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>GUILLAUME</x:v>
+      </x:c>
+      <x:c r="D8" t="str"/>
+      <x:c r="E8" t="str">
+        <x:v>responsable</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>OUI</x:v>
+      </x:c>
+      <x:c r="G8" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Ajoute les lignes modifiables avant validation
</commit_message>
<xml_diff>
--- a/outputs/modele_base_heures_engins.xlsx
+++ b/outputs/modele_base_heures_engins.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONDUCTEURS" sheetId="1" r:id="R2beb8f7a4738418a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RELEVES_MENSUELS" sheetId="2" r:id="Rae7dca00587e409f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AUDIT" sheetId="3" r:id="R1b9e2465322e4b6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONDUCTEURS" sheetId="1" r:id="R6e05a68f9f9340b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RELEVES_MENSUELS" sheetId="2" r:id="Rb8567768014445bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AUDIT" sheetId="3" r:id="Re85e50750a034501"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -445,13 +445,27 @@
       <x:c r="N1" s="2" t="str">
         <x:v>COMMENTAIRE</x:v>
       </x:c>
-      <x:c r="O1" s="2"/>
-      <x:c r="P1" s="2"/>
-      <x:c r="Q1" s="2"/>
-      <x:c r="R1" s="2"/>
-      <x:c r="S1" s="2"/>
-      <x:c r="T1" s="2"/>
-      <x:c r="U1" s="2"/>
+      <x:c r="O1" s="2" t="str">
+        <x:v>ID_LIGNE</x:v>
+      </x:c>
+      <x:c r="P1" s="2" t="str">
+        <x:v>NUM_LIGNE</x:v>
+      </x:c>
+      <x:c r="Q1" s="2" t="str">
+        <x:v>STATUT</x:v>
+      </x:c>
+      <x:c r="R1" s="2" t="str">
+        <x:v>DATE_VALIDATION</x:v>
+      </x:c>
+      <x:c r="S1" s="2" t="str">
+        <x:v>ID_RESPONSABLE</x:v>
+      </x:c>
+      <x:c r="T1" s="2" t="str">
+        <x:v>NOM_RESPONSABLE</x:v>
+      </x:c>
+      <x:c r="U1" s="2" t="str">
+        <x:v>PRENOM_RESPONSABLE</x:v>
+      </x:c>
       <x:c r="V1" s="2"/>
       <x:c r="W1" s="2"/>
       <x:c r="X1" s="2"/>

</xml_diff>

<commit_message>
Revert "Ajoute les lignes modifiables avant validation"
This reverts commit 0b8ba105415bbd0d860cd67dec1a74f8d910da59.
</commit_message>
<xml_diff>
--- a/outputs/modele_base_heures_engins.xlsx
+++ b/outputs/modele_base_heures_engins.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONDUCTEURS" sheetId="1" r:id="R6e05a68f9f9340b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RELEVES_MENSUELS" sheetId="2" r:id="Rb8567768014445bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AUDIT" sheetId="3" r:id="Re85e50750a034501"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONDUCTEURS" sheetId="1" r:id="R2beb8f7a4738418a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RELEVES_MENSUELS" sheetId="2" r:id="Rae7dca00587e409f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AUDIT" sheetId="3" r:id="R1b9e2465322e4b6c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -445,27 +445,13 @@
       <x:c r="N1" s="2" t="str">
         <x:v>COMMENTAIRE</x:v>
       </x:c>
-      <x:c r="O1" s="2" t="str">
-        <x:v>ID_LIGNE</x:v>
-      </x:c>
-      <x:c r="P1" s="2" t="str">
-        <x:v>NUM_LIGNE</x:v>
-      </x:c>
-      <x:c r="Q1" s="2" t="str">
-        <x:v>STATUT</x:v>
-      </x:c>
-      <x:c r="R1" s="2" t="str">
-        <x:v>DATE_VALIDATION</x:v>
-      </x:c>
-      <x:c r="S1" s="2" t="str">
-        <x:v>ID_RESPONSABLE</x:v>
-      </x:c>
-      <x:c r="T1" s="2" t="str">
-        <x:v>NOM_RESPONSABLE</x:v>
-      </x:c>
-      <x:c r="U1" s="2" t="str">
-        <x:v>PRENOM_RESPONSABLE</x:v>
-      </x:c>
+      <x:c r="O1" s="2"/>
+      <x:c r="P1" s="2"/>
+      <x:c r="Q1" s="2"/>
+      <x:c r="R1" s="2"/>
+      <x:c r="S1" s="2"/>
+      <x:c r="T1" s="2"/>
+      <x:c r="U1" s="2"/>
       <x:c r="V1" s="2"/>
       <x:c r="W1" s="2"/>
       <x:c r="X1" s="2"/>

</xml_diff>